<commit_message>
chore: reschedule project-progress.xlsx into 6 sprints matching sprint-plan.md
</commit_message>
<xml_diff>
--- a/project-progress.xlsx
+++ b/project-progress.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,21 +557,26 @@
           <t>Ghi chú &amp; Sản phẩm</t>
         </is>
       </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>FR-ACC-01 / TC-01, 02</t>
+          <t>Hạ tầng</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Cấu hình Firebase Auth &amp; dự án</t>
+          <t>Sửa khung: thêm gradlew, sửa icon, màu chữ dark mode, nút back</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -585,11 +591,11 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -598,14 +604,19 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>FirebaseClient.java, AuthRepository.java - google-services.json, bật Auth</t>
+          <t>gradlew, ic_launcher_background.xml, activity_main.xml, MainActivity.java</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>S1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
@@ -615,7 +626,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>Màn hình đăng nhập + kiểm tra dữ liệu</t>
+          <t>Cấu hình Firebase Auth &amp; dự án</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -630,11 +641,11 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -643,24 +654,29 @@
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>LoginActivity.java, activity_login.xml - Email/mật khẩu, xử lý lỗi</t>
+          <t>FirebaseClient.java, AuthRepository.java - google-services.json, bật Auth</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>S1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>FR-ACC-01 / TC-01</t>
+          <t>FR-ACC-01 / TC-01, 02</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Điều hướng theo vai trò sau đăng nhập</t>
+          <t>Màn hình đăng nhập bằng username/mật khẩu + kiểm tra dữ liệu</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -675,11 +691,11 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -688,7 +704,12 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>MainActivity.java, nav_graph - Truy vấn vai trò từ Firestore</t>
+          <t>LoginActivity.java, activity_login.xml - Username (email là bí danh tùy chọn), xử lý lỗi</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>S1</t>
         </is>
       </c>
     </row>
@@ -720,7 +741,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
@@ -736,21 +757,26 @@
           <t>StudentListFragment.java, StudentAdapter.java - addSnapshotListener thời gian thực</t>
         </is>
       </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>FR-USR-01..04 / TC-05..07</t>
+          <t>FR-STU-01 / TC-09</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Danh sách người dùng + thêm/sửa/xóa (Admin)</t>
+          <t>Màn hình chi tiết sinh viên</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -760,16 +786,16 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A</t>
+          <t>THÀNH VIÊN B</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -778,24 +804,29 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>UserListFragment.java, UserEditFragment.java - Phân quyền Admin quản trị</t>
+          <t>StudentDetailFragment.java, fragment_student_detail.xml - Hiển thị sinh viên và danh sách chứng chỉ</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>S1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>FR-USR-05 / TC-03, 08</t>
+          <t>FR-ACC-01 / TC-01</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Khóa/mở khóa người dùng + chặn đăng nhập</t>
+          <t>Điều hướng theo vai trò sau đăng nhập</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -823,24 +854,29 @@
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>UserRepository.java, LoginActivity.java - Chặn status Locked thời gian thực</t>
+          <t>MainActivity.java, nav_graph - Truy vấn vai trò từ Firestore</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>S2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>FR-ACC-02 / TC-04</t>
+          <t>FR-SEC / TC-07, 10, 15</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Tải ảnh đại diện cá nhân (đổi avatar)</t>
+          <t>Bảo mật Firestore &amp; Storage Rules (RBAC 3 vai trò)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -859,7 +895,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -868,7 +904,12 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>ProfileFragment.java, storage.rules - Firebase Storage avatars/{uid}.jpg</t>
+          <t>firestore.rules, storage.rules - Chặn tài khoản Locked; B review chéo</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>S2</t>
         </is>
       </c>
     </row>
@@ -916,21 +957,26 @@
           <t>StudentRepository.java, StudentEditFragment.java - Xóa sạch subcollection chứng chỉ</t>
         </is>
       </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>FR-STU-01 / TC-09</t>
+          <t>FR-USR-01..04 / TC-05..07</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Màn hình chi tiết sinh viên</t>
+          <t>Danh sách người dùng + thêm/sửa/xóa (Admin)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -940,16 +986,16 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -958,24 +1004,29 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>StudentDetailFragment.java, fragment_student_detail.xml - Hiển thị sinh viên và danh sách chứng chỉ</t>
+          <t>UserListFragment.java, UserEditFragment.java - Phân quyền Admin quản trị</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>S3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>FR-USR-06 / TC-22, 23</t>
+          <t>FR-USR-05 / TC-03, 08</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Lịch sử đăng nhập: ghi lại + xem theo người dùng</t>
+          <t>Khóa/mở khóa người dùng + chặn đăng nhập</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -990,7 +1041,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
@@ -1003,24 +1054,29 @@
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>LoginHistoryFragment.java, LoginRecordAdapter.java - Subcollection users/{uid}/loginHistory</t>
+          <t>UserRepository.java, LoginActivity.java - Chặn status Locked thời gian thực</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>S3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>FR-SEC / TC-07, 10, 15</t>
+          <t>FR-CER-01..04 / TC-14, 15</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Bảo mật Firestore &amp; Storage Rules (RBAC 3 vai trò)</t>
+          <t>CRUD chứng chỉ trong chi tiết sinh viên</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1030,12 +1086,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A</t>
+          <t>THÀNH VIÊN B</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
@@ -1048,7 +1104,12 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>firestore.rules, storage.rules - Bắt buộc B review chéo</t>
+          <t>CertificateRepository.java, CertificateEditFragment.java - Subcollection students/{id}/certificates</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>S3</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1141,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
@@ -1096,21 +1157,26 @@
           <t>StudentViewModel.java, StudentListFragment.java - Lọc realtime trên snapshot</t>
         </is>
       </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>FR-STU-06 / TC-13</t>
+          <t>FR-ACC-02 / TC-04</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Sắp xếp đa tiêu chí (Tên A-Z, GPA, Ngày sinh)</t>
+          <t>Tải ảnh đại diện cá nhân (đổi avatar)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1120,7 +1186,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1138,24 +1204,29 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>StudentViewModel.java, Vietnamese Collator - Xử lý phía client</t>
+          <t>ProfileFragment.java, storage.rules - Firebase Storage avatars/{uid}.jpg</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>FR-CER-01..04 / TC-14, 15</t>
+          <t>FR-USR-06 / TC-22, 23</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>CRUD chứng chỉ trong chi tiết sinh viên</t>
+          <t>Lịch sử đăng nhập: ghi lại + xem theo người dùng</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1165,7 +1236,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1174,7 +1245,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1183,24 +1254,29 @@
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>CertificateRepository.java, CertificateEditFragment.java - Subcollection students/{id}/certificates</t>
+          <t>LoginHistoryFragment.java, LoginRecordAdapter.java - Subcollection users/{uid}/loginHistory</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>NFR-UI</t>
+          <t>FR-STU-06 / TC-13</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Hoàn thiện UI: theme, dark mode, skeleton loading, haptics</t>
+          <t>Sắp xếp đa tiêu chí (Tên, Ngày sinh, Lớp)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1210,16 +1286,16 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A</t>
+          <t>THÀNH VIÊN B</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1228,24 +1304,29 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>ThemeManager.java, HapticFeedbackHelper.java - Material 3 design</t>
+          <t>StudentViewModel.java, Vietnamese Collator - Xử lý phía client</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>NFR-REL / TC-03</t>
+          <t>FR-IO-02 / TC-19</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Xử lý ngoại lệ, mất mạng (Offline resilience) &amp; Thông báo</t>
+          <t>Export CSV sinh viên ra bộ nhớ qua SAF (UTF-8 BOM)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1255,12 +1336,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A</t>
+          <t>THÀNH VIÊN B</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
@@ -1273,24 +1354,29 @@
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>UiNotificationHelper.java, Firestore Cache - Cache cục bộ, badge offline</t>
+          <t>CsvHelper.java, SAF Intent - Xuất file CSV mở Excel không lỗi font</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>FR-IO-01 / TC-16, 17, 24</t>
+          <t>FR-IO-04</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Import CSV sinh viên (UTF-8 BOM, chunked WriteBatch &gt;500)</t>
+          <t>Export danh sách chứng chỉ ra CSV (UTF-8 BOM)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1305,11 +1391,11 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1318,24 +1404,29 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>CsvHelper.java, ImportExportFragment.java - Xử lý batch 400 docs/lần</t>
+          <t>CsvHelper.java - Xuất chứng chỉ của sinh viên</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>S4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T18</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>FR-IO-02 / TC-19</t>
+          <t>NFR-UI</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Export CSV sinh viên ra bộ nhớ qua SAF (UTF-8 BOM)</t>
+          <t>Hoàn thiện UI: theme, dark mode, skeleton loading, haptics</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1345,16 +1436,16 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1363,24 +1454,29 @@
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>CsvHelper.java, SAF Intent - Xuất file CSV mở Excel không lỗi font</t>
+          <t>ThemeManager.java, HapticFeedbackHelper.java - Material 3 design</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>FR-IO-03 / TC-27</t>
+          <t>NFR-REL / TC-03</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Import CSV chứng chỉ theo MSSV sinh viên</t>
+          <t>Xử lý ngoại lệ, mất mạng (Offline resilience) &amp; Thông báo</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1390,12 +1486,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
@@ -1408,43 +1504,48 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>CsvHelper.java, CertificateRepository.java - Ánh xạ MSSV vào subcollection</t>
+          <t>UiNotificationHelper.java, Firestore Cache - Cache cục bộ, badge offline</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>TC-01..08, 22, 23</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Kiểm thử chéo: Thành viên B test độc lập Auth/User của A</t>
+          <t>Báo cáo (tiếng Anh): chương Firestore + phần Auth/User/Rules</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN B</t>
+          <t>THÀNH VIÊN A</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1453,29 +1554,34 @@
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>docs/test-and-setup.md (Bảng kết quả test) - B test nghiệm thu code của A</t>
+          <t>docs/final-report.md</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>TC-03, 07, 10, 15</t>
+          <t>FR-IO-01 / TC-16, 17, 24</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Kiểm thử trường hợp biên &amp; Security Rules Simulator</t>
+          <t>Import CSV sinh viên (UTF-8 BOM, chunked WriteBatch &gt;500)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1485,11 +1591,11 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1498,43 +1604,48 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>docs/test-and-setup.md - Thử truy cập trái quyền</t>
+          <t>CsvHelper.java, ImportExportFragment.java - Xử lý batch 400 docs/lần</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>TC-09..21, 24, 25, 27</t>
+          <t>FR-IO-03 / TC-27</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Kiểm thử chéo: Thành viên A test độc lập Student/CSV của B</t>
+          <t>Import CSV chứng chỉ theo MSSV sinh viên</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A</t>
+          <t>THÀNH VIÊN B</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1543,29 +1654,34 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>docs/test-and-setup.md (Bảng kết quả test) - A test nghiệm thu code của B</t>
+          <t>CsvHelper.java, CertificateRepository.java - Ánh xạ MSSV vào subcollection</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>NFR-DEMO</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Chuẩn bị dữ liệu demo, kịch bản chi tiết và thiết bị quay</t>
+          <t>Báo cáo (tiếng Anh): phần Student/Certificate/CSV</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1575,7 +1691,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
@@ -1588,29 +1704,34 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>docs/demo-script.md, sample-data/ - Cài đặt 2 máy ảo/thiết bị split-screen</t>
+          <t>docs/final-report.md</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>S5</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>NFR-DEMO</t>
+          <t>TC-09..21, 24, 25, 27</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Thuyết minh và quay video demo hoàn chỉnh (&lt;= 20 phút)</t>
+          <t>Kiểm thử chéo: Thành viên A test độc lập Student/CSV của B</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Demo</t>
+          <t>Kiểm thử</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1620,11 +1741,11 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1633,52 +1754,312 @@
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>Video demo 720p+ MP4 - A nói, B phụ trách thiết bị và góc quay</t>
+          <t>docs/test-and-setup.md (Bảng kết quả test) - A test nghiệm thu code của B</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>NFR-DEMO</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Thuyết minh và quay video demo hoàn chỉnh (&lt;= 20 phút)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>THÀNH VIÊN A</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>CẦN LÀM</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Video demo 720p+ MP4 - A nói, B phụ trách thiết bị và góc quay</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>T28</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Báo cáo</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thiện báo cáo PDF: bìa, mục lục, chú thích hình, tài liệu tham khảo</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Báo cáo</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>THÀNH VIÊN A</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>CẦN LÀM</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>Báo cáo PDF</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>T25</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>NFR-REL</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Vá lỗi cuối cùng, nghiệm thu tổng thể &amp; đóng gói bài nộp</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Kiểm thử</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>THÀNH VIÊN A</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-14</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n">
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>CẦN LÀM</t>
         </is>
       </c>
-      <c r="I26" s="11" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>Gói nộp bài hoàn chỉnh - Dry run trên máy sạch</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>TC-01..08, 22, 23</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Kiểm thử chéo: Thành viên B test độc lập Auth/User của A</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm thử</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>THÀNH VIÊN B</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>CẦN LÀM</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>docs/test-and-setup.md (Bảng kết quả test) - B test nghiệm thu code của A</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>TC-03, 07, 10, 15</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Kiểm thử trường hợp biên &amp; Security Rules Simulator</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm thử</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>THÀNH VIÊN B</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>CẦN LÀM</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>docs/test-and-setup.md - Thử truy cập trái quyền</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>NFR-DEMO</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Chuẩn bị dữ liệu demo, kịch bản chi tiết và thiết bị quay</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>THÀNH VIÊN B</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>CẦN LÀM</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>docs/demo-script.md, sample-data/ - Cài đặt 2 máy ảo/thiết bị split-screen</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>S6</t>
         </is>
       </c>
     </row>
@@ -2691,7 +3072,7 @@
       </c>
       <c r="B1" s="10" t="inlineStr">
         <is>
-          <t>THÀNH VIÊN A (Tan)</t>
+          <t>THÀNH VIÊN A (Tấn)</t>
         </is>
       </c>
       <c r="C1" s="10" t="inlineStr">

</xml_diff>